<commit_message>
Convert SWI-PRO-MET-207-007 to 207-011 (cyanide analysers) to Heritage; drop detox calibration; 207 series complete
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Register-SWI-207.xlsx
+++ b/docs/Register-SWI-207.xlsx
@@ -12,8 +12,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Keterangan" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Register 207'!$A$1:$Q$7</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Draft dan open items'!$A$1:$D$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Register 207'!$A$1:$Q$12</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Draft dan open items'!$A$1:$D$14</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -35,7 +35,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -50,6 +50,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00F8CBAD"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -84,7 +89,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -98,7 +103,10 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -469,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q7"/>
+  <dimension ref="A1:Q12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="9" customWidth="1" min="1" max="1"/>
@@ -1076,8 +1084,423 @@
         </is>
       </c>
     </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>207-007</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-207-007</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Cyanide Analyser Daily Operation and Check - 032-CA-001 and 051-CA-002</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>207 Automatic Sampling and Online Analysers</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Safety-critical</t>
+        </is>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>JSEA-PRO-MET-207-007</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2027</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="K8" s="3" t="inlineStr">
+        <is>
+          <t>To be set once the vendor manual is held.</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="M8" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="N8" s="3" t="inlineStr">
+        <is>
+          <t>Replace Filter Sock - Step 3, DRAFT (operasi harian tetap NOT FOR USE)</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>NOT FOR USE (menunggu input)</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="Q8" s="3" t="inlineStr">
+        <is>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-207-007-Cyanide-Analyser-Daily-Operation-and-Check---032-CA-001-and-051-CA-RevA.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>207-008</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-207-008</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Cyanide Analyser Calibration and Standardisation</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>207 Automatic Sampling and Online Analysers</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Safety-critical</t>
+        </is>
+      </c>
+      <c r="F9" s="3" t="inlineStr">
+        <is>
+          <t>JSEA-PRO-MET-207-008</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2027</t>
+        </is>
+      </c>
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="K9" s="3" t="inlineStr">
+        <is>
+          <t>To be set once the vendor calibration data is held.</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="M9" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="N9" s="3" t="inlineStr">
+        <is>
+          <t>Leach Analyzer Calibration - dipakai untuk kedua analyser; Detox Analyser Calibration tidak dipakai (tidak ada sirkuit detox)</t>
+        </is>
+      </c>
+      <c r="O9" s="5" t="inlineStr">
+        <is>
+          <t>DRAFT FOR REVIEW (tambahan Martabe)</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="Q9" s="3" t="inlineStr">
+        <is>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-207-008-Cyanide-Analyser-Calibration-and-Standardisation-RevA.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>207-009</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-207-009</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Cyanide Analyser Specialised Electrode Replacement and Conditioning</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>207 Automatic Sampling and Online Analysers</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Safety-critical</t>
+        </is>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>JSEA-PRO-MET-207-009</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2027</t>
+        </is>
+      </c>
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="K10" s="3" t="inlineStr">
+        <is>
+          <t>To be set once the vendor manual is held.</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M10" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="N10" s="3" t="inlineStr">
+        <is>
+          <t>Tidak ada padanan</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>NOT FOR USE (menunggu input)</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="Q10" s="3" t="inlineStr">
+        <is>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-207-009-Cyanide-Analyser-Specialised-Electrode-Replacement-and-Conditionin-RevA.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>207-010</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-207-010</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Cyanide Analyser Sample and Booster Pump Service - 032-PP-207/208 and 041-PP-2xx</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>207 Automatic Sampling and Online Analysers</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Safety-critical</t>
+        </is>
+      </c>
+      <c r="F11" s="3" t="inlineStr">
+        <is>
+          <t>JSEA-PRO-MET-207-010</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2027</t>
+        </is>
+      </c>
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="K11" s="3" t="inlineStr">
+        <is>
+          <t>To be set once the vendor manual is held.</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M11" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="N11" s="3" t="inlineStr">
+        <is>
+          <t>Tidak ada padanan</t>
+        </is>
+      </c>
+      <c r="O11" s="4" t="inlineStr">
+        <is>
+          <t>NOT FOR USE (menunggu input)</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="Q11" s="3" t="inlineStr">
+        <is>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-207-010-Cyanide-Analyser-Sample-and-Booster-Pump-Service---032-PP-207208-a-RevA.docx</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>207-011</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-207-011</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Cyanide Analyser Leak Detector and High Level Alarm Response</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>207 Automatic Sampling and Online Analysers</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Safety-critical</t>
+        </is>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>JSEA-PRO-MET-207-011</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2026</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>11/08/2027</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Processing</t>
+        </is>
+      </c>
+      <c r="K12" s="3" t="inlineStr">
+        <is>
+          <t>To be set once the alarm response is defined.</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="M12" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="N12" s="3" t="inlineStr">
+        <is>
+          <t>Tidak ada padanan</t>
+        </is>
+      </c>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>NOT FOR USE (menunggu input)</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>Sudah</t>
+        </is>
+      </c>
+      <c r="Q12" s="3" t="inlineStr">
+        <is>
+          <t>MM-4034-033-OR-03-SWI-PRO-MET-207-011-Cyanide-Analyser-Leak-Detector-and-High-Level-Alarm-Response-RevA.docx</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:Q7"/>
+  <autoFilter ref="A1:Q12"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1088,7 +1511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1098,139 +1521,315 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="5" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>No. dokumen</t>
         </is>
       </c>
-      <c r="B1" s="5" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Judul</t>
         </is>
       </c>
-      <c r="C1" s="5" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>Jenis</t>
         </is>
       </c>
-      <c r="D1" s="5" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Isi catatan</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>SWI-PRO-MET-207-001</t>
         </is>
       </c>
-      <c r="B2" s="6" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Automatic Sampler Operation and Cut Verification - IsaMill Feed 022-XM-011 and 022-XM-017</t>
         </is>
       </c>
-      <c r="C2" s="6" t="inlineStr">
+      <c r="C2" s="7" t="inlineStr">
         <is>
           <t>Catatan</t>
         </is>
       </c>
-      <c r="D2" s="6" t="inlineStr">
+      <c r="D2" s="7" t="inlineStr">
         <is>
           <t>ISSUED BUT NOT FOR USE. This document is a placeholder against the register line so the line is not empty. It cannot be used until the sampler general arrangement and cutter design are held: 022-XM-011 and 022-XM-017 are shop-fabricated with the vendor and cutter design TBA, and the mechanical equipment list shows conflicting status (NEW on one tab, FUTURE on another). The method, frequency and equipment are written when that input arrives.</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>SWI-PRO-MET-207-002</t>
         </is>
       </c>
-      <c r="B3" s="6" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Automatic Sampler Operation and Cut Verification - CIL Tails 032-XM-012</t>
         </is>
       </c>
-      <c r="C3" s="6" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>Catatan</t>
         </is>
       </c>
-      <c r="D3" s="6" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>ISSUED BUT NOT FOR USE. This document is a placeholder against the register line so the line is not empty. It cannot be used until the sampler general arrangement and cutter design are held: vendor and cutter design TBA, and the status conflicts (NEW versus FUTURE) across the equipment list tabs. The method, frequency and equipment are written when that input arrives.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>SWI-PRO-MET-207-003</t>
         </is>
       </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Automatic Sampler Operation and Cut Verification - Metal Adsorption Tails 041-XM-013</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="C4" s="7" t="inlineStr">
         <is>
           <t>Catatan</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="D4" s="7" t="inlineStr">
         <is>
           <t>ISSUED BUT NOT FOR USE. This document is a placeholder against the register line so the line is not empty. It cannot be used until the sampler general arrangement and cutter design are held: vendor and cutter design TBA. The method, frequency and equipment are written when that input arrives.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>SWI-PRO-MET-207-004</t>
         </is>
       </c>
-      <c r="B5" s="6" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Automatic Sampler Operation and Cut Verification - Final Tails 051-XM-014</t>
         </is>
       </c>
-      <c r="C5" s="6" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Catatan</t>
         </is>
       </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>ISSUED BUT NOT FOR USE. This document is a placeholder against the register line so the line is not empty. It cannot be used until the sampler general arrangement and cutter design are held: vendor and cutter design TBA, and no P&amp;ID reference is given on the equipment list. The method, frequency and equipment are written when that input arrives.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>SWI-PRO-MET-207-005</t>
         </is>
       </c>
-      <c r="B6" s="6" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Automatic Sampler Cleaning, Unblocking and Cutter Wear Check</t>
         </is>
       </c>
-      <c r="C6" s="6" t="inlineStr">
+      <c r="C6" s="7" t="inlineStr">
         <is>
           <t>Catatan</t>
         </is>
       </c>
-      <c r="D6" s="6" t="inlineStr">
+      <c r="D6" s="7" t="inlineStr">
         <is>
           <t>ISSUED BUT NOT FOR USE. This document is a placeholder against the register line so the line is not empty. It cannot be used until the sampler general arrangement and cutter design are held: no source is held for any of the five samplers. The method, frequency and equipment are written when that input arrives.</t>
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-207-007</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Cyanide Analyser Daily Operation and Check - 032-CA-001 and 051-CA-002</t>
+        </is>
+      </c>
+      <c r="C7" s="7" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="D7" s="7" t="inlineStr">
+        <is>
+          <t>Draft for review: the filter sock replacement (Step 3) is taken from the Martabe work instruction Replace Filter Sock (DOC-3-MET-PMC-WIN-00091, undated), written for the Martabe analyser filter probe. JSEA-PRO-MET-207-007 must be updated for the added hazard before it is used.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-207-007</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="inlineStr">
+        <is>
+          <t>Cyanide Analyser Daily Operation and Check - 032-CA-001 and 051-CA-002</t>
+        </is>
+      </c>
+      <c r="C8" s="7" t="inlineStr">
+        <is>
+          <t>Catatan</t>
+        </is>
+      </c>
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>ISSUED BUT NOT FOR USE. The daily operation and check (Step 2) cannot be used until the named input arrives: the Molycop Cynoprobe v3 WAD vendor manual is not held and OS-040_B Cyanide Analyser is still open. The method, frequency and equipment are written when that input arrives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-207-007</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Cyanide Analyser Daily Operation and Check - 032-CA-001 and 051-CA-002</t>
+        </is>
+      </c>
+      <c r="C9" s="7" t="inlineStr">
+        <is>
+          <t>Open items</t>
+        </is>
+      </c>
+      <c r="D9" s="7" t="inlineStr">
+        <is>
+          <t>Open items: (1) confirm the equivalent filter probe and parts on 032-CA-001 and 051-CA-002, and whether these analysers have HCl dosing; (2) the source works from photographs that are not carried here - confirm the filtrate line arrangement for the flush; (3) the source gives no frequency for the filter sock change.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-207-008</t>
+        </is>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>Cyanide Analyser Calibration and Standardisation</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>Draft</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>Draft for review: the calibration method (Steps 2 to 5) is taken from the Martabe work instruction Leach Analyzer Calibration (DOC-3-MET-PMC-WIN-00126-IE, v1.0, 25/12/2024) and applies to both analysers. The Martabe Detox Analyser Calibration is not used: there is no detox circuit at Mt. Morgan - the ReCYN circuit follows CIL. JSEA-PRO-MET-207-008 must be updated for the added hazard before this instruction is approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-207-008</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Cyanide Analyser Calibration and Standardisation</t>
+        </is>
+      </c>
+      <c r="C11" s="7" t="inlineStr">
+        <is>
+          <t>Open items</t>
+        </is>
+      </c>
+      <c r="D11" s="7" t="inlineStr">
+        <is>
+          <t>Open items: (1) the source calibrates free NaCN only, with the WAD calibration box NOT ticked; the Mt. Morgan analysers read free and WAD cyanide, so the WAD calibration must be set from the Cynoprobe v3 WAD calibration data, which is not held; (2) standards - the Indonesian source gives 250, 500 and 700 ppm NaCN, its English copy 30, 250 and 500 ppm (taken from the detox instruction); confirm the leach standards and set the range for 051-CA-002 on the ReCYN circuit; (3) the source verification pH range of 9 to 11 reaches below the 10.5 cyanide safety limit; (4) the troubleshooting guide for critical errors is an attachment that was not received; (5) confirm the cyanide-bearing return point for leftover standard (the source says the leach tank) and the record folders.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-207-009</t>
+        </is>
+      </c>
+      <c r="B12" s="7" t="inlineStr">
+        <is>
+          <t>Cyanide Analyser Specialised Electrode Replacement and Conditioning</t>
+        </is>
+      </c>
+      <c r="C12" s="7" t="inlineStr">
+        <is>
+          <t>Catatan</t>
+        </is>
+      </c>
+      <c r="D12" s="7" t="inlineStr">
+        <is>
+          <t>ISSUED BUT NOT FOR USE. This document is a placeholder against the register line so the line is not empty. It cannot be used until the named input arrives: the Molycop Cynoprobe vendor manual is not held, and no procedure is held for the Mintex 3000366 and 3000330 electrodes. The method, frequency and equipment are written when that input arrives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-207-010</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Cyanide Analyser Sample and Booster Pump Service - 032-PP-207/208 and 041-PP-2xx</t>
+        </is>
+      </c>
+      <c r="C13" s="7" t="inlineStr">
+        <is>
+          <t>Catatan</t>
+        </is>
+      </c>
+      <c r="D13" s="7" t="inlineStr">
+        <is>
+          <t>ISSUED BUT NOT FOR USE. This document is a placeholder against the register line so the line is not empty. It cannot be used until the named input arrives: the Vender Dura 10 pump manual is not held (the pumps are listed as part of the Molycop package). The method, frequency and equipment are written when that input arrives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>SWI-PRO-MET-207-011</t>
+        </is>
+      </c>
+      <c r="B14" s="7" t="inlineStr">
+        <is>
+          <t>Cyanide Analyser Leak Detector and High Level Alarm Response</t>
+        </is>
+      </c>
+      <c r="C14" s="7" t="inlineStr">
+        <is>
+          <t>Catatan</t>
+        </is>
+      </c>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>ISSUED BUT NOT FOR USE. This document is a placeholder against the register line so the line is not empty. It cannot be used until the named input arrives: the Azbil HPQ-D12 leak detector and E&amp;H FTL31 level switch are vendor scope and no alarm response is held. The method, frequency and equipment are written when that input arrives.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:D6"/>
+  <autoFilter ref="A1:D14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1248,49 +1847,49 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="6" t="inlineStr">
-        <is>
-          <t>Register seri 207 Automatic Samplers and Analysers (6 dokumen dalam format Heritage).</t>
+      <c r="A1" s="7" t="inlineStr">
+        <is>
+          <t>Register seri 207 Automatic Samplers and Analysers (11 dokumen dalam format Heritage).</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="6" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>Data dibaca langsung dari Part 1 dan Part 2 tiap dokumen (judul, tanggal, owner, JSEA ID, area, frekuensi).</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="6" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>Klasifikasi dan padanan Martabe diambil dari docs/Matriks-Rujukan-Martabe.xlsx dan docs/Tabel-SWI-vs-Martabe.xlsx, ditimpa oleh keputusan review bila ada. Format Heritage tidak memuat kolom klasifikasi, jadi klasifikasi hanya ada di register.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="6" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>Jumlah step dan halaman dihitung dari render dokumen (LibreOffice); halaman bisa sedikit berbeda di Microsoft Word.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="6" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>Status isi: Final = tanpa tambahan Martabe terbuka; DRAFT FOR REVIEW = ada tambahan Martabe yang menunggu JSEA; Catatan = ada catatan yang perlu ditindaklanjuti.</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>Sheet "Draft dan open items" memuat paragraf draft, catatan, temuan safety-critical, dan open items di Description of work.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="6" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>Referensi register: HM-MMM-WHS-REG-XXX-R00-SWI-SWMS, tab SWI-MET.</t>
         </is>

</xml_diff>

<commit_message>
207-008: map Martabe detox analyser calibration to ReCYN tailing analyser 051-CA-002
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01UHnSDEBA56GANs2gfXuK2P
</commit_message>
<xml_diff>
--- a/docs/Register-SWI-207.xlsx
+++ b/docs/Register-SWI-207.xlsx
@@ -1224,14 +1224,14 @@
         </is>
       </c>
       <c r="L9" s="2" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="M9" s="2" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="N9" s="3" t="inlineStr">
         <is>
-          <t>Leach Analyzer Calibration - dipakai untuk kedua analyser; Detox Analyser Calibration tidak dipakai (tidak ada sirkuit detox)</t>
+          <t>Leach Analyzer Calibration untuk 032-CA-001; Detox Analyser Calibration dipetakan ke analyser ReCYN tailing 051-CA-002</t>
         </is>
       </c>
       <c r="O9" s="5" t="inlineStr">
@@ -1736,7 +1736,7 @@
       </c>
       <c r="D10" s="7" t="inlineStr">
         <is>
-          <t>Draft for review: the calibration method (Steps 2 to 5) is taken from the Martabe work instruction Leach Analyzer Calibration (DOC-3-MET-PMC-WIN-00126-IE, v1.0, 25/12/2024) and applies to both analysers. The Martabe Detox Analyser Calibration is not used: there is no detox circuit at Mt. Morgan - the ReCYN circuit follows CIL. JSEA-PRO-MET-207-008 must be updated for the added hazard before this instruction is approved.</t>
+          <t>Draft for review: Steps 2 to 5 (032-CA-001) are taken from the Martabe work instruction Leach Analyzer Calibration (DOC-3-MET-PMC-WIN-00126-IE). Step 6 (051-CA-002) is taken from the Martabe Detox Analyser Calibration (DOC-3-MET-PMC-WIN-00117-IE): Mt. Morgan has no detox circuit - the ReCYN circuit follows CIL - so the Martabe detox analyser maps to the ReCYN tailing analyser 051-CA-002. Both v1.0, 25/12/2024. JSEA-PRO-MET-207-008 must be updated for the added hazards before this instruction is approved.</t>
         </is>
       </c>
     </row>
@@ -1758,7 +1758,7 @@
       </c>
       <c r="D11" s="7" t="inlineStr">
         <is>
-          <t>Open items: (1) the source calibrates free NaCN only, with the WAD calibration box NOT ticked; the Mt. Morgan analysers read free and WAD cyanide, so the WAD calibration must be set from the Cynoprobe v3 WAD calibration data, which is not held; (2) standards - the Indonesian source gives 250, 500 and 700 ppm NaCN, its English copy 30, 250 and 500 ppm (taken from the detox instruction); confirm the leach standards and set the range for 051-CA-002 on the ReCYN circuit; (3) the source verification pH range of 9 to 11 reaches below the 10.5 cyanide safety limit; (4) the troubleshooting guide for critical errors is an attachment that was not received; (5) confirm the cyanide-bearing return point for leftover standard (the source says the leach tank) and the record folders.</t>
+          <t>Open items: (1) the source calibrates free NaCN only, with the WAD calibration box NOT ticked; the Mt. Morgan analysers read free and WAD cyanide, so the WAD calibration must be set from the Cynoprobe v3 WAD calibration data, which is not held; (2) standards for 032-CA-001 - the Indonesian source gives 250, 500 and 700 ppm NaCN, its English copy 30, 250 and 500 ppm; confirm; (3) standards for 051-CA-002 - the source materials list gives 30, 125 and 250 ppm, the steps give 30, 250 and 500 ppm; confirm against the ReCYN tailing range; (4) verification pH ranges in the source (9 to 11 for the leach analyser, 6 to 9 for the detox stream) reach below the 10.5 cyanide safety limit; confirm the range for each stream, in particular the ReCYN tailing; (5) the troubleshooting guide for critical errors is an attachment that was not received; (6) confirm the cyanide-bearing return point for leftover standard (the source says the leach tank) and the record folders.</t>
         </is>
       </c>
     </row>

</xml_diff>